<commit_message>
Match building control notices citing ABP case numbers without prefix
Commencement notices written as 22-313124 or 313124-22 were not linked to
the SHD; Raheen (ABP-313124-22, 384 units) is under construction since
April 2024, not unstarted. Report and GeoPackage regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/delivery_study/Limerick_Delivery_Study_Data.xlsx
+++ b/limerick_pipeline/delivery_study/Limerick_Delivery_Study_Data.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7021" uniqueCount="1032">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7011" uniqueCount="1032">
   <si>
     <t xml:space="preserve">Limerick residential delivery study – data companion</t>
   </si>
@@ -3844,19 +3844,19 @@
         <v>1287</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>571</v>
+        <v>955</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3998,19 +3998,19 @@
         <v>1958</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1454</v>
+        <v>1838</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4458,19 +4458,19 @@
         <v>5444</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3689</v>
+        <v>4073</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F4" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>67</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4586,19 +4586,19 @@
         <v>5444</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>3689</v>
+        <v>4073</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F3" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>67</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4842,16 +4842,16 @@
         <v>1282</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>847</v>
+        <v>1231</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>0.8</v>
@@ -5197,10 +5197,10 @@
         <v>98</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>749</v>
+        <v>1133</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1073</v>
+        <v>689</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>0</v>
@@ -5429,7 +5429,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>1.8</v>
@@ -5578,19 +5578,19 @@
         <v>154</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>131</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>99</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>83</v>
@@ -5931,7 +5931,7 @@
         <v>990</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>180</v>
@@ -5946,13 +5946,13 @@
         <v>262</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>1641</v>
+        <v>1257</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>10</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>4200</v>
+        <v>3816</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24218,7 +24218,7 @@
         <v>257</v>
       </c>
       <c r="R165" s="2" t="s">
-        <v>75</v>
+        <v>103</v>
       </c>
       <c r="S165" s="6" t="n">
         <v>44645</v>
@@ -24235,13 +24235,17 @@
       <c r="W165" s="6" t="n">
         <v>48394</v>
       </c>
-      <c r="X165" s="6"/>
-      <c r="Y165" s="2"/>
+      <c r="X165" s="6" t="n">
+        <v>45406</v>
+      </c>
+      <c r="Y165" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="Z165" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA165" s="2" t="n">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="AB165" s="6"/>
       <c r="AC165" s="2" t="n">
@@ -24253,7 +24257,9 @@
       <c r="AE165" s="7" t="n">
         <v>0.265571526351814</v>
       </c>
-      <c r="AF165" s="7"/>
+      <c r="AF165" s="7" t="n">
+        <v>1.81793292265572</v>
+      </c>
       <c r="AG165" s="7"/>
       <c r="AH165" s="7"/>
       <c r="AI165" s="2" t="s">
@@ -35352,7 +35358,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P112"/>
+  <dimension ref="A1:P111"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="1" style="0" width="12"/>
@@ -39748,67 +39754,65 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>629</v>
+        <v>865</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>630</v>
+        <v>866</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>631</v>
+        <v>867</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>283</v>
+        <v>851</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>632</v>
+        <v>851</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>633</v>
+        <v>69</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>384</v>
+        <v>31</v>
       </c>
       <c r="I92" s="2" t="s">
-        <v>286</v>
+        <v>91</v>
       </c>
       <c r="J92" s="2" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="K92" s="6" t="n">
-        <v>44742</v>
-      </c>
-      <c r="L92" s="6" t="n">
-        <v>48394</v>
-      </c>
+        <v>44967</v>
+      </c>
+      <c r="L92" s="2"/>
       <c r="M92" s="2" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="N92" s="2" t="s">
-        <v>257</v>
+        <v>74</v>
       </c>
       <c r="O92" s="6" t="n">
-        <v>45649.5284866898</v>
+        <v>44979.4748903125</v>
       </c>
       <c r="P92" s="2"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>865</v>
+        <v>93</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>866</v>
+        <v>65</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>867</v>
+        <v>94</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>851</v>
+        <v>67</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>851</v>
+        <v>68</v>
       </c>
       <c r="F93" s="2" t="s">
         <v>69</v>
@@ -39823,10 +39827,10 @@
         <v>91</v>
       </c>
       <c r="J93" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K93" s="6" t="n">
-        <v>44967</v>
+        <v>43857</v>
       </c>
       <c r="L93" s="2"/>
       <c r="M93" s="2" t="s">
@@ -39836,34 +39840,34 @@
         <v>74</v>
       </c>
       <c r="O93" s="6" t="n">
-        <v>44979.4748903125</v>
+        <v>43781.6000934838</v>
       </c>
       <c r="P93" s="2"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>93</v>
+        <v>522</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>65</v>
+        <v>523</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>94</v>
+        <v>524</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>68</v>
+        <v>467</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>69</v>
+        <v>514</v>
       </c>
       <c r="G94" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="I94" s="2" t="s">
         <v>91</v>
@@ -39872,7 +39876,7 @@
         <v>95</v>
       </c>
       <c r="K94" s="6" t="n">
-        <v>43857</v>
+        <v>43740</v>
       </c>
       <c r="L94" s="2"/>
       <c r="M94" s="2" t="s">
@@ -39882,43 +39886,43 @@
         <v>74</v>
       </c>
       <c r="O94" s="6" t="n">
-        <v>43781.6000934838</v>
+        <v>44998.4572684838</v>
       </c>
       <c r="P94" s="2"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>522</v>
+        <v>736</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>523</v>
+        <v>676</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>524</v>
+        <v>737</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>82</v>
+        <v>678</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>467</v>
+        <v>632</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>514</v>
+        <v>69</v>
       </c>
       <c r="G95" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I95" s="2" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="J95" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="K95" s="6" t="n">
-        <v>43740</v>
+        <v>44950</v>
       </c>
       <c r="L95" s="2"/>
       <c r="M95" s="2" t="s">
@@ -39928,34 +39932,32 @@
         <v>74</v>
       </c>
       <c r="O95" s="6" t="n">
-        <v>44998.4572684838</v>
+        <v>44987.4668805903</v>
       </c>
       <c r="P95" s="2"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="2" t="s">
-        <v>736</v>
-      </c>
+      <c r="A96" s="2"/>
       <c r="B96" s="2" t="s">
-        <v>676</v>
+        <v>544</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>737</v>
+        <v>545</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>678</v>
+        <v>283</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>632</v>
+        <v>467</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>69</v>
+        <v>514</v>
       </c>
       <c r="G96" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I96" s="2" t="s">
         <v>118</v>
@@ -39963,96 +39965,98 @@
       <c r="J96" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="K96" s="6" t="n">
-        <v>44950</v>
-      </c>
+      <c r="K96" s="2"/>
       <c r="L96" s="2"/>
       <c r="M96" s="2" t="s">
         <v>991</v>
       </c>
       <c r="N96" s="2" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="O96" s="6" t="n">
-        <v>44987.4668805903</v>
+        <v>46203.387381794</v>
       </c>
       <c r="P96" s="2"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="2"/>
+      <c r="A97" s="2" t="s">
+        <v>767</v>
+      </c>
       <c r="B97" s="2" t="s">
-        <v>544</v>
+        <v>744</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>545</v>
+        <v>768</v>
       </c>
       <c r="D97" s="2" t="s">
         <v>283</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>467</v>
+        <v>632</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>514</v>
+        <v>633</v>
       </c>
       <c r="G97" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="I97" s="2" t="s">
         <v>118</v>
       </c>
       <c r="J97" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="K97" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="K97" s="6" t="n">
+        <v>45677</v>
+      </c>
       <c r="L97" s="2"/>
       <c r="M97" s="2" t="s">
         <v>991</v>
       </c>
       <c r="N97" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="O97" s="6" t="n">
-        <v>46203.387381794</v>
+        <v>45693.580934456</v>
       </c>
       <c r="P97" s="2"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>767</v>
+        <v>871</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>744</v>
+        <v>873</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>768</v>
+        <v>874</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>283</v>
+        <v>82</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>632</v>
+        <v>851</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>633</v>
+        <v>69</v>
       </c>
       <c r="G98" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I98" s="2" t="s">
         <v>118</v>
       </c>
       <c r="J98" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="K98" s="6" t="n">
-        <v>45677</v>
+        <v>44614</v>
       </c>
       <c r="L98" s="2"/>
       <c r="M98" s="2" t="s">
@@ -40062,25 +40066,25 @@
         <v>74</v>
       </c>
       <c r="O98" s="6" t="n">
-        <v>45693.580934456</v>
+        <v>44526.4160490741</v>
       </c>
       <c r="P98" s="2"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>871</v>
+        <v>402</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>873</v>
+        <v>403</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>874</v>
+        <v>404</v>
       </c>
       <c r="D99" s="2" t="s">
         <v>82</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>851</v>
+        <v>284</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>69</v>
@@ -40089,16 +40093,16 @@
         <v>97</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I99" s="2" t="s">
         <v>118</v>
       </c>
       <c r="J99" s="2" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="K99" s="6" t="n">
-        <v>44614</v>
+        <v>43811</v>
       </c>
       <c r="L99" s="2"/>
       <c r="M99" s="2" t="s">
@@ -40108,31 +40112,31 @@
         <v>74</v>
       </c>
       <c r="O99" s="6" t="n">
-        <v>44526.4160490741</v>
+        <v>43780.5776577546</v>
       </c>
       <c r="P99" s="2"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>402</v>
+        <v>886</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>403</v>
+        <v>887</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>404</v>
+        <v>888</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>82</v>
+        <v>855</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>284</v>
+        <v>851</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>69</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="H100" s="2" t="n">
         <v>12</v>
@@ -40143,98 +40147,98 @@
       <c r="J100" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="K100" s="6" t="n">
-        <v>43811</v>
-      </c>
+      <c r="K100" s="2"/>
       <c r="L100" s="2"/>
       <c r="M100" s="2" t="s">
         <v>991</v>
       </c>
       <c r="N100" s="2" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="O100" s="6" t="n">
-        <v>43780.5776577546</v>
+        <v>46181.3513474884</v>
       </c>
       <c r="P100" s="2"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>886</v>
+        <v>809</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>887</v>
+        <v>741</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>888</v>
+        <v>810</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>855</v>
+        <v>82</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>851</v>
+        <v>632</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>69</v>
+        <v>400</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I101" s="2" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="J101" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="K101" s="2"/>
+        <v>92</v>
+      </c>
+      <c r="K101" s="6" t="n">
+        <v>44659</v>
+      </c>
       <c r="L101" s="2"/>
       <c r="M101" s="2" t="s">
         <v>991</v>
       </c>
       <c r="N101" s="2" t="s">
-        <v>182</v>
+        <v>74</v>
       </c>
       <c r="O101" s="6" t="n">
-        <v>46181.3513474884</v>
+        <v>44917.5037965278</v>
       </c>
       <c r="P101" s="2"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>809</v>
+        <v>906</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>741</v>
+        <v>907</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>810</v>
+        <v>908</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>82</v>
+        <v>855</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>632</v>
+        <v>851</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>400</v>
+        <v>69</v>
       </c>
       <c r="G102" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I102" s="2" t="s">
         <v>139</v>
       </c>
       <c r="J102" s="2" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="K102" s="6" t="n">
-        <v>44659</v>
+        <v>43368</v>
       </c>
       <c r="L102" s="2"/>
       <c r="M102" s="2" t="s">
@@ -40244,74 +40248,72 @@
         <v>74</v>
       </c>
       <c r="O102" s="6" t="n">
-        <v>44917.5037965278</v>
+        <v>43346.6208667824</v>
       </c>
       <c r="P102" s="2"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>906</v>
+        <v>433</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>907</v>
+        <v>434</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>908</v>
+        <v>435</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>855</v>
+        <v>283</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>851</v>
+        <v>284</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>69</v>
+        <v>295</v>
       </c>
       <c r="G103" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I103" s="2" t="s">
         <v>139</v>
       </c>
       <c r="J103" s="2" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="K103" s="6" t="n">
-        <v>43368</v>
+        <v>46006</v>
       </c>
       <c r="L103" s="2"/>
       <c r="M103" s="2" t="s">
         <v>991</v>
       </c>
       <c r="N103" s="2" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="O103" s="6" t="n">
-        <v>43346.6208667824</v>
+        <v>46148.4278019329</v>
       </c>
       <c r="P103" s="2"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="B104" s="2" t="s">
-        <v>434</v>
-      </c>
+        <v>614</v>
+      </c>
+      <c r="B104" s="2"/>
       <c r="C104" s="2" t="s">
-        <v>435</v>
+        <v>615</v>
       </c>
       <c r="D104" s="2" t="s">
         <v>283</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>284</v>
+        <v>467</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>295</v>
+        <v>468</v>
       </c>
       <c r="G104" s="2" t="s">
         <v>97</v>
@@ -40323,80 +40325,82 @@
         <v>139</v>
       </c>
       <c r="J104" s="2" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="K104" s="6" t="n">
-        <v>46006</v>
+        <v>43264</v>
       </c>
       <c r="L104" s="2"/>
       <c r="M104" s="2" t="s">
         <v>991</v>
       </c>
       <c r="N104" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="O104" s="6" t="n">
-        <v>46148.4278019329</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="O104" s="2"/>
       <c r="P104" s="2"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B105" s="2"/>
+        <v>918</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>919</v>
+      </c>
       <c r="C105" s="2" t="s">
-        <v>615</v>
+        <v>920</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>283</v>
+        <v>82</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>467</v>
+        <v>851</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>468</v>
+        <v>69</v>
       </c>
       <c r="G105" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I105" s="2" t="s">
         <v>139</v>
       </c>
       <c r="J105" s="2" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="K105" s="6" t="n">
-        <v>43264</v>
+        <v>45335</v>
       </c>
       <c r="L105" s="2"/>
       <c r="M105" s="2" t="s">
         <v>991</v>
       </c>
       <c r="N105" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="O105" s="2"/>
+        <v>182</v>
+      </c>
+      <c r="O105" s="6" t="n">
+        <v>45912.3574854514</v>
+      </c>
       <c r="P105" s="2"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>918</v>
+        <v>271</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>919</v>
+        <v>272</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>920</v>
+        <v>273</v>
       </c>
       <c r="D106" s="2" t="s">
         <v>82</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>851</v>
+        <v>158</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>69</v>
@@ -40405,16 +40409,16 @@
         <v>97</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I106" s="2" t="s">
         <v>139</v>
       </c>
       <c r="J106" s="2" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="K106" s="6" t="n">
-        <v>45335</v>
+        <v>42256</v>
       </c>
       <c r="L106" s="2"/>
       <c r="M106" s="2" t="s">
@@ -40424,72 +40428,68 @@
         <v>182</v>
       </c>
       <c r="O106" s="6" t="n">
-        <v>45912.3574854514</v>
+        <v>42807.4205058681</v>
       </c>
       <c r="P106" s="2"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="2" t="s">
-        <v>271</v>
-      </c>
+      <c r="A107" s="2"/>
       <c r="B107" s="2" t="s">
-        <v>272</v>
+        <v>624</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>273</v>
+        <v>625</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>82</v>
+        <v>283</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>158</v>
+        <v>467</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>69</v>
+        <v>468</v>
       </c>
       <c r="G107" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I107" s="2" t="s">
-        <v>139</v>
+        <v>92</v>
       </c>
       <c r="J107" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="K107" s="6" t="n">
-        <v>42256</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="K107" s="2"/>
       <c r="L107" s="2"/>
       <c r="M107" s="2" t="s">
         <v>991</v>
       </c>
       <c r="N107" s="2" t="s">
-        <v>182</v>
+        <v>84</v>
       </c>
       <c r="O107" s="6" t="n">
-        <v>42807.4205058681</v>
+        <v>46213.41174375</v>
       </c>
       <c r="P107" s="2"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2"/>
       <c r="B108" s="2" t="s">
-        <v>624</v>
+        <v>924</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>625</v>
+        <v>925</v>
       </c>
       <c r="D108" s="2" t="s">
         <v>283</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>467</v>
+        <v>92</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>468</v>
+        <v>92</v>
       </c>
       <c r="G108" s="2" t="s">
         <v>97</v>
@@ -40509,20 +40509,20 @@
         <v>991</v>
       </c>
       <c r="N108" s="2" t="s">
-        <v>84</v>
+        <v>182</v>
       </c>
       <c r="O108" s="6" t="n">
-        <v>46213.41174375</v>
+        <v>46079.3742551273</v>
       </c>
       <c r="P108" s="2"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2"/>
       <c r="B109" s="2" t="s">
-        <v>924</v>
+        <v>926</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>925</v>
+        <v>927</v>
       </c>
       <c r="D109" s="2" t="s">
         <v>283</v>
@@ -40536,9 +40536,7 @@
       <c r="G109" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="H109" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="H109" s="2"/>
       <c r="I109" s="2" t="s">
         <v>92</v>
       </c>
@@ -40554,52 +40552,32 @@
         <v>182</v>
       </c>
       <c r="O109" s="6" t="n">
-        <v>46079.3742551273</v>
+        <v>46190.3328899306</v>
       </c>
       <c r="P109" s="2"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2"/>
-      <c r="B110" s="2" t="s">
-        <v>926</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>927</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F110" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G110" s="2" t="s">
-        <v>97</v>
-      </c>
+      <c r="B110" s="2"/>
+      <c r="C110" s="2"/>
+      <c r="D110" s="2"/>
+      <c r="E110" s="2"/>
+      <c r="F110" s="2"/>
+      <c r="G110" s="2"/>
       <c r="H110" s="2"/>
-      <c r="I110" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="J110" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="I110" s="2"/>
+      <c r="J110" s="2"/>
       <c r="K110" s="2"/>
       <c r="L110" s="2"/>
-      <c r="M110" s="2" t="s">
-        <v>991</v>
-      </c>
-      <c r="N110" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="O110" s="6" t="n">
-        <v>46190.3328899306</v>
-      </c>
+      <c r="M110" s="2"/>
+      <c r="N110" s="2"/>
+      <c r="O110" s="2"/>
       <c r="P110" s="2"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="2"/>
+      <c r="A111" s="11" t="s">
+        <v>937</v>
+      </c>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
       <c r="D111" s="2"/>
@@ -40615,26 +40593,6 @@
       <c r="N111" s="2"/>
       <c r="O111" s="2"/>
       <c r="P111" s="2"/>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="11" t="s">
-        <v>937</v>
-      </c>
-      <c r="B112" s="2"/>
-      <c r="C112" s="2"/>
-      <c r="D112" s="2"/>
-      <c r="E112" s="2"/>
-      <c r="F112" s="2"/>
-      <c r="G112" s="2"/>
-      <c r="H112" s="2"/>
-      <c r="I112" s="2"/>
-      <c r="J112" s="2"/>
-      <c r="K112" s="2"/>
-      <c r="L112" s="2"/>
-      <c r="M112" s="2"/>
-      <c r="N112" s="2"/>
-      <c r="O112" s="2"/>
-      <c r="P112" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -40765,7 +40723,7 @@
         <v>1402</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1223</v>
+        <v>1607</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>350</v>
@@ -41097,10 +41055,10 @@
         <v>1006</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>5551</v>
+        <v>5167</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41274,7 +41232,7 @@
         <v>1021</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -41554,11 +41512,11 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$L$2:$L$267,$A7,Schemes!$R$2:$R$267,"Under construction")</f>
-        <v>1126</v>
+        <v>1510</v>
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$L$2:$L$267,$A7,Schemes!$R$2:$R$267,"Not started – permission live")</f>
-        <v>3341</v>
+        <v>2957</v>
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$L$2:$L$267,$A7,Schemes!$R$2:$R$267,"Not started – past expiry")</f>
@@ -41583,11 +41541,11 @@
       </c>
       <c r="D8" s="10" t="n">
         <f aca="false">SUM(D3:D7)</f>
-        <v>3680</v>
+        <v>4064</v>
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">SUM(E3:E7)</f>
-        <v>5551</v>
+        <v>5167</v>
       </c>
       <c r="F8" s="10" t="n">
         <f aca="false">SUM(F3:F7)</f>
@@ -41722,11 +41680,11 @@
       </c>
       <c r="D15" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$G$2:$G$267,$A15,Schemes!$R$2:$R$267,"Under construction")</f>
-        <v>1578</v>
+        <v>1962</v>
       </c>
       <c r="E15" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$G$2:$G$267,$A15,Schemes!$R$2:$R$267,"Not started – permission live")</f>
-        <v>1973</v>
+        <v>1589</v>
       </c>
       <c r="F15" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$G$2:$G$267,$A15,Schemes!$R$2:$R$267,"Not started – past expiry")</f>
@@ -42064,11 +42022,11 @@
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$H$2:$H$267,$A29,Schemes!$R$2:$R$267,"Under construction")</f>
-        <v>749</v>
+        <v>1133</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$H$2:$H$267,$A29,Schemes!$R$2:$R$267,"Not started – permission live")</f>
-        <v>1073</v>
+        <v>689</v>
       </c>
       <c r="F29" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$H$2:$H$267,$A29,Schemes!$R$2:$R$267,"Not started – past expiry")</f>
@@ -42261,11 +42219,11 @@
       </c>
       <c r="D38" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$P$2:$P$267,$A38,Schemes!$R$2:$R$267,"Under construction")</f>
-        <v>2963</v>
+        <v>3347</v>
       </c>
       <c r="E38" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$P$2:$P$267,$A38,Schemes!$R$2:$R$267,"Not started – permission live")</f>
-        <v>5015</v>
+        <v>4631</v>
       </c>
       <c r="F38" s="9" t="n">
         <f aca="false">SUMIFS(Schemes!$K$2:$K$267,Schemes!$P$2:$P$267,$A38,Schemes!$R$2:$R$267,"Not started – past expiry")</f>
@@ -42428,10 +42386,10 @@
         <v>438</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1126</v>
+        <v>1510</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>3341</v>
+        <v>2957</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>137</v>
@@ -42451,10 +42409,10 @@
         <v>1275</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>3680</v>
+        <v>4064</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>5551</v>
+        <v>5167</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>311</v>
@@ -42722,16 +42680,16 @@
         <v>0.7</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>3</v>
@@ -42760,7 +42718,7 @@
         <v>0.9</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0.7</v>
@@ -42959,19 +42917,19 @@
         <v>14</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>12</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>9</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>8</v>
@@ -42992,7 +42950,7 @@
         <v>208</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>182</v>
@@ -43004,7 +42962,7 @@
         <v>143</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>119</v>
@@ -43161,16 +43119,16 @@
         <v>2517</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1700</v>
+        <v>2084</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>1.4</v>
@@ -43445,19 +43403,19 @@
         <v>2250</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1564</v>
+        <v>1948</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43573,19 +43531,19 @@
         <v>2875</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2004</v>
+        <v>2388</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>